<commit_message>
Keep one topic in topics list spreadsheet
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -557,298 +557,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Imported (undated)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist (category idea)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Kids' chapter book series (ages 6 to 9)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Kids' chapter book series (ages 6 to 9): text-only, repeatable structure, series loyalty; price $2.99 to $4.99.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Imported (undated)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist (category idea)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Bedtime story collections</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Bedtime story collections: short self-contained stories in themed volumes; steady gift and routine buyers.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Imported (undated)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist (category idea)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Early readers (ages 4 to 7)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Early readers (ages 4 to 7): controlled vocabulary; recurring character; check reading level before publishing.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Imported (undated)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist (category idea)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Large-print puzzle books</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Large-print puzzle books: no writing-quality risk; low price and heavy competition.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Imported (undated)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist (category idea)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Narrow practical how-to guides</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Narrow practical how-to guides: one reader, one problem; every fact must be verified; avoid medical, financial, and legal advice.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Halden Point Cozy Mystery Series: Book 1, Slack Water</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>When the relief lighthouse keeper of Halden Point is found dead at the foot of the tower, the coroner calls it a fall on the wet steps. Nell Ardery, a widowed tea-room owner who runs the cafe below the lighthouse, doesn't believe it. The tide tables and the lighthouse logbook don't agree about when the tide turned, and someone has rewritten one page of the log. Nell works through the village's small circle of suspects: the ferry secretary who keeps the timetables, the lifeboat volunteer who lost money from the fund, a painter who rents the old signal room, and the vicar's sister who knows everyone's secrets. Each clue depends on the tides, so the answer is fair and checkable by the reader. The story is warm and witty, with no on-page violence, no sexual content, and no profanity, and it ends with the village restored and a hook for Book 2.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Mystery, Thriller &amp; Suspense &gt; Women Sleuths (also check the Cozy subcategory in the KDP category picker; the exact browse node was not confirmed).</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Text-only ebook, reflowable. Series: yes, planned as a 3 to 5 book series with a recurring cast and setting.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before the delivery fee, which is negligible for a text-only file.</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>about 210 to 230 pages</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>55,000 to 60,000 words</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Adult cozy mystery readers (women 35 to 70 are the core) who read on Kindle Unlimited and want a comforting, puzzle-driven story with a recurring cast and a sense of place. The book delivers the feeling of being part of a small town and the satisfaction of solving the clue before the sleuth does.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>1. 1. Slack Water: Nell finds the body at dawn, with the lighthouse door unlocked and a torch still burning.
-2. 2. The Tide Table: the coroner rules a fall; Nell notices the logbook page is wrong.
-3. 3. The Keeper's Widow: Nell visits the dead keeper's wife and learns he had been worried about money.
-4. 4. Teacups and Suspects: the tea room becomes the village's gossip hub; the first suspects are introduced.
-5. 5. The Ferry Timetable: a second look at the ferry schedule shows a gap that fits the timeline.
-6. 6. A Lie in the Signal Room: the painter's alibi fails, but he has his own secret.
-7. 7. Lifeboat Accounts: the fund's missing money points to a suspect nobody expected.
-8. 8. Low Tide Confessions: Nell finds the rewritten page hidden in a second logbook.
-9. 9. The Storm Log: the confrontation at the tower during a squall; the fair-play clue is revealed.
-10. 10. Full Tide: the culprit is caught; the village starts to heal.
-11. 11. Epilogue: Next Tide: a new letter arrives at the tea room and sets up Book 2.</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>1. Slack Water: A Halden Point Cozy Mystery
-2. The Keeper's Ledger: A Lighthouse Cove Mystery, Book 1
-3. Tide Tables and Tea: A Halden Point Cozy Mystery</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>1. cozy mystery lighthouse
-2. small town women sleuth mystery
-3. cozy mystery series ebook
-4. amateur sleuth coastal village
-5. cozy murder mystery Kindle Unlimited
-6. lighthouse mystery novel
-7. tea room cozy mystery</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>label: ESTIMATE. No sales data was verified. These are planning assumptions, not sourced figures.; reasoning: A new indie cozy mystery with no reviews is assumed to sell slowly at first. Sales are expected to rise as Books 2 and 3 publish and KU reads accumulate. The assumed price is $4.99 at a 70% royalty, or about $3.49 per sale. KU pages are at the $0.00482 per page rate from profitable.app.; scenarios: [{'case': 'Conservative', 'sales_per_month': 20, 'kenp_pages_per_month': 4000, 'estimated_monthly_revenue_usd': 88}, {'case': 'Mid', 'sales_per_month': 40, 'kenp_pages_per_month': 10000, 'estimated_monthly_revenue_usd': 186}, {'case': 'Optimistic (series of 3+ books)', 'sales_per_month': 100, 'kenp_pages_per_month': 25000, 'estimated_monthly_revenue_usd': 466}]; revenue_formula: sales x $3.49 + KENP pages x $0.00482</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>1. Quality: AI prose may be flat, and AI-written mystery clues often fail the fair-play test. Mitigation: outline the clue chain before drafting, have a human check every clue against the tide table, and do a full human read-through before upload.
-2. Competition: the cozy mystery shelf is crowded and dominated by indie series. Mitigation: the tide-table and logbook clue mechanism is a distinct hook; differentiate covers and blurbs; publish Books 2 and 3 quickly.
-3. Policy: KDP requires AI-generated text to be disclosed (private checkbox). Reported upload caps (3 per day) may slow a catalog build. Mitigation: disclose correctly, pace uploads, and never claim human authorship in marketing.
-4. Originality: cozy mysteries share tropes. Mitigation: do not copy existing series names, characters, or plots; check new titles against the Kindle store before publishing.
-5. Demand is not verified: Amazon Best Sellers pages were blocked during research. Mitigation: pull rank data for three to five comparable cozy mysteries before committing to Book 2.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q8"/>
+  <autoFilter ref="A1:Q2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove category column from topics list
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$P$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -498,67 +498,62 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Format</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Price (USD)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Price (USD)</t>
+          <t>Royalty</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Royalty</t>
+          <t>Pages</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Pages</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Words</t>
+          <t>Target reader</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Target reader</t>
+          <t>Chapter outline</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Chapter outline</t>
+          <t>Title options</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Title options</t>
+          <t>KDP keywords</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>KDP keywords</t>
+          <t>Sales estimate (ESTIMATE)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Sales estimate (ESTIMATE)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Risks</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q2"/>
+  <autoFilter ref="A1:P2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore category column in topics list
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,14 +448,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -493,67 +493,72 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Price (USD)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Royalty</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Pages</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Words</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Target reader</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Chapter outline</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Title options</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>KDP keywords</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Sales estimate (ESTIMATE)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Risks</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:Q2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Bakery on Cutter Street romance topic to topics spreadsheet
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,112 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Selected - not yet used</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>The Bakery on Cutter Street, Book 1: Flour, Frost and a Second Chance</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Small Town (verify the exact browse node in the KDP category picker; not confirmed).</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Hannah Brooks has just returned to Cutter Street, the small Ohio town she left at eighteen, to take over her late grandmother's bakery. The shop is in debt, the oven is temperamental, and the one person who can fix the ovens is Eli Carver, the town's grumpy contractor who was her first crush and her grandmother's favorite fixer of everything. As they rebuild the bakery together, Hannah has to decide whether to sell the shop to a developer who has made a generous offer or keep it and the life she is starting to like. Eli has his own reasons for staying out of town politics. The story is warm, funny and romantic, with a close-knit cast of bakers, regulars and a dog who visits the shop every morning. It has no explicit sexual content, no profanity and no on-page violence. It ends with the bakery open, the developer defeated by the town and a hook for Book 2.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Text-only ebook, reflowable. Series: yes, planned as a 3 to 4 book series set on Cutter Street with a recurring cast.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>3.99</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee, which is negligible for a text-only file.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>about 180 to 200 pages</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>50,000 to 55,000 words</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Adult readers of sweet small-town romance who read on Kindle Unlimited, mostly women 30 to 60. They want a comforting love story with a clear happy ending and a strong sense of place.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>1. Opening Day: Hannah returns to the bakery and finds the oven dead and the cash box nearly empty.
+2. The Man With the Wrench: Eli Carver arrives, unwilling, to look at the oven, and they clash over the repair bill.
+3. Sourdough and Old Promises: Hannah finds her grandmother's notes and the history between her and Eli.
+4. The Developer's Offer: a generous offer arrives, and the town begins to take sides.
+5. Saturday Market: the bakery's first market stall brings regulars back and a new complication.
+6. Late Nights in the Kitchen: Hannah and Eli work late, and the tension turns into friendship.
+7. The Town Meeting: Eli is asked to speak against the developer, and he refuses.
+8. The Winter Harvest: a storm damages the shop, and the town helps rebuild it.
+9. A Letter From the Past: Hannah learns why her grandmother never sold the shop.
+10. Open for Business: Hannah chooses the bakery and tells Eli how she feels.
+11. Epilogue: First Snow: the shop is full, and a new visitor sets up Book 2.</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>The Bakery on Cutter Street
+Flour, Frost and a Second Chance
+Sourdough on Cutter Street</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>small town romance
+bakery romance
+sweet romance series
+contemporary romance kindle unlimited
+clean romance adult</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ESTIMATE. No sales data was verified. These are planning assumptions, not sourced figures. Price and royalty come from the plan; the per-page KENP rate is a third-party estimate. A new small-town romance with no reviews is assumed to sell slowly. Sales are expected to rise as Books 2 and 3 publish and Kindle Unlimited reads build. Monthly revenue = sales x $2.79 + KENP pages x $0.00482. The category is crowded, so the conservative case is the planning case. Scenarios: Conservative: 10 sales/month, 1,500 KENP pages/month, about $35/month; Mid: 25 sales/month, 6,000 KENP pages/month, about $99/month; Optimistic (series of 3+ books): 60 sales/month, 15,000 KENP pages/month, about $240/month. Formula: sales x $2.79 + KENP pages x $0.00482</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Crowded category with large publishers: differentiate with the bakery setting, a clear series hook and a strong cover.
+AI-drafted romance can read flat: the manuscript needs a human editor focused on dialogue and chemistry before upload.
+Category and keyword choices are not verified in the KDP picker: check before publishing.
+No demand data: run a small test with a single Book 1 price before committing to Book 2.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Extend topics spreadsheet filter to include new topic row
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics'!$A$1:$Q$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -664,7 +664,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q2"/>
+  <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix robot pipeline: topic sync, run log, KDP tracker
- scripts/sync_topics.py copies new log topics into topics-list.xlsx as Selected,
  so the picker can find them. Holds Halden Point until the owner decides.
- scripts/log_run.py and reports/run-log.json: every robot records one line per run.
- Ready to publish/kdp-drafts.json: Kindle-4 draft tracker.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,166 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The Second Act Workbook: A 30-Day Guided Reflection Journal for Starting Over After Work</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Self-Help &gt; Personal Transformation (browse node not confirmed; verify the exact path in the KDP category picker, and check Self-Help &gt; Aging or Retirement if offered).</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Retirement, a layoff, a career change or a grown-up child leaving home can leave a reader with a full calendar and no clear sense of who they are outside their old role. The Second Act Workbook is a guided reflection journal with a short prompt for each day of a 30-day course, grouped into ten chapters. Readers start by naming what their work gave them, then log how their days actually go, list the skills they have that matter outside a job, map the relationships they want more of, and run two-week trials of new activities such as volunteering, a class or a walking group. The workbook avoids clinical language and makes no medical or financial recommendations: it contains no investment, pension or budgeting prompts, and it points readers to a professional when a question needs one. It ends with a one-page plan and a 90-day review sheet, so the reader leaves with a direction rather than a pep talk.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Text-only, reflowable ebook with fillable prompts laid out as lined text blocks (no images). Series: optional. Planned as a companion to a later title on caregiving transitions only if this book sells.</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before any delivery fee, which is small for a text-only file.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>about 115 to 125 Kindle pages (estimate, from 14,000 to 16,000 words, with prompts and space for notes)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>14,000 to 16,000 words</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Adults aged about 55 to 70 who have recently retired, been made redundant or stepped back from full-time work, and who want a structured, private way to reflect on their next chapter. Secondary readers are adult children and partners buying a gift for someone in transition. The book solves the problem of 'who am I now that my job is over?' without offering medical or financial advice.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1. The Badge in the Drawer: naming what work gave you, besides a paycheck.
+2. The Inventory of Days: a one-week log of how time actually goes, hour by hour.
+3. Skills Beyond the Job: listing abilities that matter in a volunteer group, a family or a neighbourhood.
+4. The People Who Count: mapping relationships and choosing where to spend more time.
+5. Curiosity Reopened: rediscovering interests dropped in the busy years.
+6. Two-Week Trials: a menu of small experiments such as a class, a choir, a garden plot or a book club.
+7. Naming the Friction: prompts for the fears and habits that hold a reader back, with no diagnosis or therapy advice.
+8. Structure Without a Schedule: building flexible weekly rhythms.
+9. Saying Yes, Saying No: boundaries with family, old colleagues and well-meaning friends.
+10. Your Second Act Plan: a one-page plan, then a 90-day review sheet.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>The Second Act Workbook: A 30-Day Guided Journal for Starting Over After Work
+Who Are You Now? A 30-Day Reflection Workbook for Life After Work
+The Next Chapter Journal: Thirty Days to Your Second Act</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Arts &amp; Photography &gt; Music &gt; Instruction &amp; Study (browse node not confirmed; verify in the KDP category picker. Education &amp; Teaching is the alternative to check).</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Many adults who took up piano, guitar or singing after years away stall when they reach printed music. Read Sheet Music Fast is a text-based workbook that builds staff reading one step at a time: the staff and clefs, note names on the treble and bass clef, note values, rests, ties and dots, key signatures and the circle of fifths, then a first simple melody and finally two-hand reading on the grand staff. Each chapter ends with short exercises and an answer key, and a 20-minute daily practice plan closes the book. The book deliberately avoids theory for its own sake and teaches only what a reader needs to play or sing the next page. Music diagrams are made with a music engraving tool, not generated by AI, and every notation example and answer key is checked by a human musician before publication.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Reflowable text-only ebook with notation figures, each drawn with a music engraving tool and exported as an image. The figures are not AI-generated, so they do not need image disclosure, but the disclosure review should confirm this. Series: planned as Book 1 of a two-book set (Book 2 covers rhythm and sight-reading).</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee. The delivery fee is small for a text-only file with a few image files.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>about 100 to 110 Kindle pages (estimate, from 11,000 to 13,000 words plus exercises and an answer key)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>11,000 to 13,000 words</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Adults who play piano, keyboard, guitar or sing in a choir, have a basic sense of the instrument and want to read music properly. Typical readers are aged 25 to 65 and studying alone, with no regular teacher. The book solves the problem of 'I can play by ear, but I can't read the notes on the page'.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1. Why Sheet Music Looks Hard, and Why It Isn't: the five lines, the four spaces, and a first look at a score.
+2. Clefs and Staffs: the treble and bass clefs, ledger lines and where middle C sits.
+3. Treble Clef Note Names: reading notes on the lines and spaces with mnemonics and drills.
+4. Bass Clef Note Names: the same method, with the bass clef's own landmarks.
+5. Note Values: whole, half, quarter and eighth notes, and how they add up to a beat.
+6. Rests, Ties and Dots: silence, holds and dotted values in simple rhythms.
+7. Key Signatures and the Circle of Fifths: sharps, flats and how they change the notes.
+8. Reading Your First Melody: a step-by-step walk through a short tune.
+9. Two Hands on the Grand Staff: reading both clefs at once, with a warm-up exercise.
+10. A 20-Minute Practice Plan: daily routines and a way to measure progress.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers
+Reading the Notes: Book 1, Staff, Clefs and Rhythm for Adult Beginners
+The Printed Page: Learn to Read Music, Step by Step, at Your Own Pace</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kindle-2: ebook package for The Second Act Workbook
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Selected</t>
+          <t>Used - 2026-10-18</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -741,7 +741,6 @@
 The Next Chapter Journal: Thirty Days to Your Second Act</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -821,7 +820,6 @@
 The Printed Page: Learn to Read Music, Step by Step, at Your Own Pace</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>

</xml_diff>

<commit_message>
Remove The Second Act Workbook: book folder, topic, used mark, spreadsheet row, run-log entry
Owner request: delete this ebook and all its content.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -674,132 +674,53 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Used - 2026-10-18</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Second Act Workbook: A 30-Day Guided Reflection Journal for Starting Over After Work</t>
+          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Self-Help &gt; Personal Transformation (browse node not confirmed; verify the exact path in the KDP category picker, and check Self-Help &gt; Aging or Retirement if offered).</t>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Arts &amp; Photography &gt; Music &gt; Instruction &amp; Study (browse node not confirmed; verify in the KDP category picker. Education &amp; Teaching is the alternative to check).</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Retirement, a layoff, a career change or a grown-up child leaving home can leave a reader with a full calendar and no clear sense of who they are outside their old role. The Second Act Workbook is a guided reflection journal with a short prompt for each day of a 30-day course, grouped into ten chapters. Readers start by naming what their work gave them, then log how their days actually go, list the skills they have that matter outside a job, map the relationships they want more of, and run two-week trials of new activities such as volunteering, a class or a walking group. The workbook avoids clinical language and makes no medical or financial recommendations: it contains no investment, pension or budgeting prompts, and it points readers to a professional when a question needs one. It ends with a one-page plan and a 90-day review sheet, so the reader leaves with a direction rather than a pep talk.</t>
+          <t>Many adults who took up piano, guitar or singing after years away stall when they reach printed music. Read Sheet Music Fast is a text-based workbook that builds staff reading one step at a time: the staff and clefs, note names on the treble and bass clef, note values, rests, ties and dots, key signatures and the circle of fifths, then a first simple melody and finally two-hand reading on the grand staff. Each chapter ends with short exercises and an answer key, and a 20-minute daily practice plan closes the book. The book deliberately avoids theory for its own sake and teaches only what a reader needs to play or sing the next page. Music diagrams are made with a music engraving tool, not generated by AI, and every notation example and answer key is checked by a human musician before publication.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Text-only, reflowable ebook with fillable prompts laid out as lined text blocks (no images). Series: optional. Planned as a companion to a later title on caregiving transitions only if this book sells.</t>
+          <t>Reflowable text-only ebook with notation figures, each drawn with a music engraving tool and exported as an image. The figures are not AI-generated, so they do not need image disclosure, but the disclosure review should confirm this. Series: planned as Book 1 of a two-book set (Book 2 covers rhythm and sight-reading).</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>4.99</v>
+        <v>3.99</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before any delivery fee, which is small for a text-only file.</t>
+          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee. The delivery fee is small for a text-only file with a few image files.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>about 115 to 125 Kindle pages (estimate, from 14,000 to 16,000 words, with prompts and space for notes)</t>
+          <t>about 100 to 110 Kindle pages (estimate, from 11,000 to 13,000 words plus exercises and an answer key)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>14,000 to 16,000 words</t>
+          <t>11,000 to 13,000 words</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Adults aged about 55 to 70 who have recently retired, been made redundant or stepped back from full-time work, and who want a structured, private way to reflect on their next chapter. Secondary readers are adult children and partners buying a gift for someone in transition. The book solves the problem of 'who am I now that my job is over?' without offering medical or financial advice.</t>
+          <t>Adults who play piano, keyboard, guitar or sing in a choir, have a basic sense of the instrument and want to read music properly. Typical readers are aged 25 to 65 and studying alone, with no regular teacher. The book solves the problem of 'I can play by ear, but I can't read the notes on the page'.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t>1. The Badge in the Drawer: naming what work gave you, besides a paycheck.
-2. The Inventory of Days: a one-week log of how time actually goes, hour by hour.
-3. Skills Beyond the Job: listing abilities that matter in a volunteer group, a family or a neighbourhood.
-4. The People Who Count: mapping relationships and choosing where to spend more time.
-5. Curiosity Reopened: rediscovering interests dropped in the busy years.
-6. Two-Week Trials: a menu of small experiments such as a class, a choir, a garden plot or a book club.
-7. Naming the Friction: prompts for the fears and habits that hold a reader back, with no diagnosis or therapy advice.
-8. Structure Without a Schedule: building flexible weekly rhythms.
-9. Saying Yes, Saying No: boundaries with family, old colleagues and well-meaning friends.
-10. Your Second Act Plan: a one-page plan, then a 90-day review sheet.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>The Second Act Workbook: A 30-Day Guided Journal for Starting Over After Work
-Who Are You Now? A 30-Day Reflection Workbook for Life After Work
-The Next Chapter Journal: Thirty Days to Your Second Act</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Arts &amp; Photography &gt; Music &gt; Instruction &amp; Study (browse node not confirmed; verify in the KDP category picker. Education &amp; Teaching is the alternative to check).</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Many adults who took up piano, guitar or singing after years away stall when they reach printed music. Read Sheet Music Fast is a text-based workbook that builds staff reading one step at a time: the staff and clefs, note names on the treble and bass clef, note values, rests, ties and dots, key signatures and the circle of fifths, then a first simple melody and finally two-hand reading on the grand staff. Each chapter ends with short exercises and an answer key, and a 20-minute daily practice plan closes the book. The book deliberately avoids theory for its own sake and teaches only what a reader needs to play or sing the next page. Music diagrams are made with a music engraving tool, not generated by AI, and every notation example and answer key is checked by a human musician before publication.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Reflowable text-only ebook with notation figures, each drawn with a music engraving tool and exported as an image. The figures are not AI-generated, so they do not need image disclosure, but the disclosure review should confirm this. Series: planned as Book 1 of a two-book set (Book 2 covers rhythm and sight-reading).</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee. The delivery fee is small for a text-only file with a few image files.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>about 100 to 110 Kindle pages (estimate, from 11,000 to 13,000 words plus exercises and an answer key)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>11,000 to 13,000 words</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Adults who play piano, keyboard, guitar or sing in a choir, have a basic sense of the instrument and want to read music properly. Typical readers are aged 25 to 65 and studying alone, with no regular teacher. The book solves the problem of 'I can play by ear, but I can't read the notes on the page'.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
         <is>
           <t>1. Why Sheet Music Looks Hard, and Why It Isn't: the five lines, the four spaces, and a first look at a score.
 2. Clefs and Staffs: the treble and bass clefs, ledger lines and where middle C sits.
@@ -813,7 +734,7 @@
 10. A 20-Minute Practice Plan: daily routines and a way to measure progress.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers
 Reading the Notes: Book 1, Staff, Clefs and Rhythm for Adult Beginners

</xml_diff>

<commit_message>
Kindle-1: 2 topics for 2026-10-18
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -742,6 +742,215 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Romantic Comedy | Kindle Store &gt; Kindle eBooks &gt; Mystery, Thriller &amp; Suspense &gt; Cozy Mystery</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>When the groom's grandfather's gold signet ring disappears an hour before the Wexford and Adair wedding at the Tern Harbor inn, wedding planner Winnie Dorsey has to find it before the reception starts. By midnight the best man is dead on the boathouse dock, the police call it a fall, and Winnie does not believe it. Her search runs through a nervous bridal party, a jealous florist, a harbor full of gossip and Jonah Pell, the harbor master who has been her favorite irritation since high school and who is now the only person willing to check the tide logs with her. The book is a sweet, funny cozy romantic mystery with no explicit sexual content, no profanity and no on-page violence. The clues are fair, the romance is slow and earned, and the ending solves the murder, saves the wedding and leaves Winnie and Jonah with a first date. It is Book 1 of a series set in Tern Harbor, with a recurring cast of vendors, inn staff and a boat-shop cat.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>text-only</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>about 200 to 225 pages (estimate, about 275 words a page)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>55,000 to 62,000 words</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Adult readers of romantic comedy and cozy mysteries who read on Kindle Unlimited, mostly women aged 28 to 55 who want a mystery with a love story and a happy ending.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1. The Ring Goes Missing: Winnie finds the signet ring gone one hour before the ceremony.
+2. The Harbor Master Says No: Jonah refuses to help, then changes his mind when the best man's car turns up at the dock.
+3. Something Borrowed: Winnie interviews the bridal party and finds three people with a reason to lie.
+4. The Boathouse at Midnight: the best man is found dead on the boathouse dock.
+5. Tide Tables and Lies: Winnie and Jonah compare the tide logs with the coroner's report.
+6. The Florist's Secret: a jealous florist and an old feud complicate the timeline.
+7. Rehearsal Dinner: a toast reveals a debt and a motive.
+8. Slow Dancing in the Rain: a quiet evening turns the banter into something real.
+9. The Ring Is Found: the signet ring turns up somewhere nobody expected.
+10. Vows: the killer is exposed and the wedding goes on.
+11. First Date: a short epilogue, a first date and a hook for Book 2.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1
+Ring Bearer: A Cozy Romantic Mystery
+Something Borrowed, Someone Buried: A Tern Harbor Mystery</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>cozy romantic mystery
+romantic comedy mystery novel
+wedding planner cozy mystery
+small town cozy mystery romance
+funny cozy mystery kindle unlimited
+sweet romantic mystery series
+cozy mystery romance book one</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>ESTIMATE. No sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045, the midpoint of $0.0040 to $0.0045 for 2026. Monthly revenue = sales x $2.79 + KENP pages x $0.0045. Conservative: 10 sales and 1,500 KENP pages a month, about $35. Mid: 25 sales and 6,000 pages, about $97. Optimistic (series of three or more books): 60 sales and 15,000 pages, about $235.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Crowded category with large publishers. Differentiate with the wedding-planner hook and a clear series arc.
+AI-drafted romance can read flat. The chemistry and dialogue need a human editor before upload.
+Cozy mystery clues must be fair and the timeline must hold. Run a timeline check against the tide logs in review.
+Cozy Mystery is adjacent to Women Sleuths, which the 2026-10-17 topic used. Confirm the owner is comfortable with this pairing.
+No sales data for this premise. Test one price before committing to Book 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Crafts, Hobbies &amp; Home &gt; Crafts | Kindle Store &gt; Kindle eBooks &gt; Travel</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Many adults who want a travel journal stop after the first page because they believe they cannot draw. Pocket Sketchbook is a 30-day beginner's guide to sketching on trips. It teaches the few skills that make a quick drawing of a street, a cafe or a harbor recognizable: seeing shapes before details, drawing simple buildings with one or two vanishing points, sketching people as quick gestures, and adding color in ten minutes with a limited palette. Each chapter ends with a practice task of 15 to 20 minutes that can be done at home before the trip. The book is practical rather than a talent test, and it makes no medical, financial or legal claims. Because it is text-only, every drawing step is described in plain words, and every technique claim is checked against a named source listed in the metadata before publication. Destination facts are left out so the book does not go stale.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>text-only</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before any delivery fee.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>about 55 to 65 Kindle pages (estimate, from 12,000 to 14,000 words at about 220 words a page)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>12,000 to 14,000 words</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Adults aged about 35 to 70 who travel, want a sketching habit and believe they cannot draw. They buy Kindle guides for a hobby and want something they can read before a trip and keep in a bag.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1. Why Travel Sketching Works: the goal is a memory, not a masterpiece.
+2. Pack Light: a pen, a small brush, a travel palette and a pocket sketchbook.
+3. Ten Lines a Day: warm-up drills for line, shape and proportion.
+4. Seeing Before Drawing: contour and gesture drawing, step by step.
+5. Buildings Without a Ruler: simple perspective with one and two vanishing points.
+6. People in Motion: sketching figures as quick shapes and capturing a street scene.
+7. Color in Ten Minutes: a limited palette and quick washes.
+8. Writing in the Margins: captions, dates and simple travel journaling.
+9. Sketching in Public: onlookers, weather and time limits.
+10. Thirty Days Before the Trip: a practice plan and a final review sheet.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road
+Draw Where You Are: Travel Sketching for Adults Who Think They Can't Draw
+The Little Travel Sketchbook: Thirty Days of Simple Drawing and Color</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>travel sketching for beginners
+sketchbook guide for adult beginners
+travel journaling drawing guide
+learn to sketch on vacation
+beginner drawing guide for adults
+pocket sketchbook drawing tips
+drawing for adults who cannot draw</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>ESTIMATE. No Kindle sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045 (midpoint of $0.0040 to $0.0045 for 2026). Monthly revenue = sales x $3.49 + KENP pages x $0.0045. Conservative: 8 sales and 1,000 KENP pages a month, about $32. Mid: 20 sales and 4,000 pages, about $88. Optimistic (a follow-up destination title): 45 sales and 10,000 pages, about $202.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Text-only means drawing steps are explained in words without example images. The instructions must be clear enough to follow without pictures; a figure-based edition would need a different format.
+The urban sketching space has established named series. Do not use series names or the Urban Sketching Handbook title.
+Technique claims need named sources in metadata.json. Any unsourced technique claim is removed.
+Amazon Best Sellers and KDP help pages were not available, so the niche has no direct Kindle sales data.
+Destination facts are excluded to avoid stale information.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Owner: delete Read Sheet Music Fast topic (log, spreadsheet)
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -679,22 +679,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers</t>
+          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Arts &amp; Photography &gt; Music &gt; Instruction &amp; Study (browse node not confirmed; verify in the KDP category picker. Education &amp; Teaching is the alternative to check).</t>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Romantic Comedy | Kindle Store &gt; Kindle eBooks &gt; Mystery, Thriller &amp; Suspense &gt; Cozy Mystery</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Many adults who took up piano, guitar or singing after years away stall when they reach printed music. Read Sheet Music Fast is a text-based workbook that builds staff reading one step at a time: the staff and clefs, note names on the treble and bass clef, note values, rests, ties and dots, key signatures and the circle of fifths, then a first simple melody and finally two-hand reading on the grand staff. Each chapter ends with short exercises and an answer key, and a 20-minute daily practice plan closes the book. The book deliberately avoids theory for its own sake and teaches only what a reader needs to play or sing the next page. Music diagrams are made with a music engraving tool, not generated by AI, and every notation example and answer key is checked by a human musician before publication.</t>
+          <t>When the groom's grandfather's gold signet ring disappears an hour before the Wexford and Adair wedding at the Tern Harbor inn, wedding planner Winnie Dorsey has to find it before the reception starts. By midnight the best man is dead on the boathouse dock, the police call it a fall, and Winnie does not believe it. Her search runs through a nervous bridal party, a jealous florist, a harbor full of gossip and Jonah Pell, the harbor master who has been her favorite irritation since high school and who is now the only person willing to check the tide logs with her. The book is a sweet, funny cozy romantic mystery with no explicit sexual content, no profanity and no on-page violence. The clues are fair, the romance is slow and earned, and the ending solves the murder, saves the wedding and leaves Winnie and Jonah with a first date. It is Book 1 of a series set in Tern Harbor, with a recurring cast of vendors, inn staff and a boat-shop cat.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Reflowable text-only ebook with notation figures, each drawn with a music engraving tool and exported as an image. The figures are not AI-generated, so they do not need image disclosure, but the disclosure review should confirm this. Series: planned as Book 1 of a two-book set (Book 2 covers rhythm and sight-reading).</t>
+          <t>text-only</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -702,104 +702,25 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee. The delivery fee is small for a text-only file with a few image files.</t>
+          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>about 100 to 110 Kindle pages (estimate, from 11,000 to 13,000 words plus exercises and an answer key)</t>
+          <t>about 200 to 225 pages (estimate, about 275 words a page)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>11,000 to 13,000 words</t>
+          <t>55,000 to 62,000 words</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Adults who play piano, keyboard, guitar or sing in a choir, have a basic sense of the instrument and want to read music properly. Typical readers are aged 25 to 65 and studying alone, with no regular teacher. The book solves the problem of 'I can play by ear, but I can't read the notes on the page'.</t>
+          <t>Adult readers of romantic comedy and cozy mysteries who read on Kindle Unlimited, mostly women aged 28 to 55 who want a mystery with a love story and a happy ending.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t>1. Why Sheet Music Looks Hard, and Why It Isn't: the five lines, the four spaces, and a first look at a score.
-2. Clefs and Staffs: the treble and bass clefs, ledger lines and where middle C sits.
-3. Treble Clef Note Names: reading notes on the lines and spaces with mnemonics and drills.
-4. Bass Clef Note Names: the same method, with the bass clef's own landmarks.
-5. Note Values: whole, half, quarter and eighth notes, and how they add up to a beat.
-6. Rests, Ties and Dots: silence, holds and dotted values in simple rhythms.
-7. Key Signatures and the Circle of Fifths: sharps, flats and how they change the notes.
-8. Reading Your First Melody: a step-by-step walk through a short tune.
-9. Two Hands on the Grand Staff: reading both clefs at once, with a warm-up exercise.
-10. A 20-Minute Practice Plan: daily routines and a way to measure progress.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Read Sheet Music Fast: A Beginner's Workbook for Adult Pianists and Singers
-Reading the Notes: Book 1, Staff, Clefs and Rhythm for Adult Beginners
-The Printed Page: Learn to Read Music, Step by Step, at Your Own Pace</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Romantic Comedy | Kindle Store &gt; Kindle eBooks &gt; Mystery, Thriller &amp; Suspense &gt; Cozy Mystery</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>When the groom's grandfather's gold signet ring disappears an hour before the Wexford and Adair wedding at the Tern Harbor inn, wedding planner Winnie Dorsey has to find it before the reception starts. By midnight the best man is dead on the boathouse dock, the police call it a fall, and Winnie does not believe it. Her search runs through a nervous bridal party, a jealous florist, a harbor full of gossip and Jonah Pell, the harbor master who has been her favorite irritation since high school and who is now the only person willing to check the tide logs with her. The book is a sweet, funny cozy romantic mystery with no explicit sexual content, no profanity and no on-page violence. The clues are fair, the romance is slow and earned, and the ending solves the murder, saves the wedding and leaves Winnie and Jonah with a first date. It is Book 1 of a series set in Tern Harbor, with a recurring cast of vendors, inn staff and a boat-shop cat.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>text-only</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>about 200 to 225 pages (estimate, about 275 words a page)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>55,000 to 62,000 words</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Adult readers of romantic comedy and cozy mysteries who read on Kindle Unlimited, mostly women aged 28 to 55 who want a mystery with a love story and a happy ending.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
         <is>
           <t>1. The Ring Goes Missing: Winnie finds the signet ring gone one hour before the ceremony.
 2. The Harbor Master Says No: Jonah refuses to help, then changes his mind when the best man's car turns up at the dock.
@@ -814,14 +735,14 @@
 11. First Date: a short epilogue, a first date and a hook for Book 2.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1
 Ring Bearer: A Cozy Romantic Mystery
 Something Borrowed, Someone Buried: A Tern Harbor Mystery</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>cozy romantic mystery
 romantic comedy mystery novel
@@ -832,12 +753,12 @@
 cozy mystery romance book one</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>ESTIMATE. No sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045, the midpoint of $0.0040 to $0.0045 for 2026. Monthly revenue = sales x $2.79 + KENP pages x $0.0045. Conservative: 10 sales and 1,500 KENP pages a month, about $35. Mid: 25 sales and 6,000 pages, about $97. Optimistic (series of three or more books): 60 sales and 15,000 pages, about $235.</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Crowded category with large publishers. Differentiate with the wedding-planner hook and a clear series arc.
 AI-drafted romance can read flat. The chemistry and dialogue need a human editor before upload.
@@ -847,64 +768,64 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>6</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Selected</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Kindle Store &gt; Kindle eBooks &gt; Crafts, Hobbies &amp; Home &gt; Crafts | Kindle Store &gt; Kindle eBooks &gt; Travel</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Many adults who want a travel journal stop after the first page because they believe they cannot draw. Pocket Sketchbook is a 30-day beginner's guide to sketching on trips. It teaches the few skills that make a quick drawing of a street, a cafe or a harbor recognizable: seeing shapes before details, drawing simple buildings with one or two vanishing points, sketching people as quick gestures, and adding color in ten minutes with a limited palette. Each chapter ends with a practice task of 15 to 20 minutes that can be done at home before the trip. The book is practical rather than a talent test, and it makes no medical, financial or legal claims. Because it is text-only, every drawing step is described in plain words, and every technique claim is checked against a named source listed in the metadata before publication. Destination facts are left out so the book does not go stale.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>text-only</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H4" t="n">
         <v>4.99</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before any delivery fee.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>about 55 to 65 Kindle pages (estimate, from 12,000 to 14,000 words at about 220 words a page)</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>12,000 to 14,000 words</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Adults aged about 35 to 70 who travel, want a sketching habit and believe they cannot draw. They buy Kindle guides for a hobby and want something they can read before a trip and keep in a bag.</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>1. Why Travel Sketching Works: the goal is a memory, not a masterpiece.
 2. Pack Light: a pen, a small brush, a travel palette and a pocket sketchbook.
@@ -918,14 +839,14 @@
 10. Thirty Days Before the Trip: a practice plan and a final review sheet.</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road
 Draw Where You Are: Travel Sketching for Adults Who Think They Can't Draw
 The Little Travel Sketchbook: Thirty Days of Simple Drawing and Color</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>travel sketching for beginners
 sketchbook guide for adult beginners
@@ -936,12 +857,12 @@
 drawing for adults who cannot draw</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>ESTIMATE. No Kindle sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045 (midpoint of $0.0040 to $0.0045 for 2026). Monthly revenue = sales x $3.49 + KENP pages x $0.0045. Conservative: 8 sales and 1,000 KENP pages a month, about $32. Mid: 20 sales and 4,000 pages, about $88. Optimistic (a follow-up destination title): 45 sales and 10,000 pages, about $202.</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Text-only means drawing steps are explained in words without example images. The instructions must be clear enough to follow without pictures; a figure-based edition would need a different format.
 The urban sketching space has established named series. Do not use series names or the Urban Sketching Handbook title.

</xml_diff>

<commit_message>
Owner: delete all topics created by the robots today (Nobody Brings a Shovel; Pocket Sketchbook). Bakery kept (owner request, published).
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -663,215 +663,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Romantic Comedy | Kindle Store &gt; Kindle eBooks &gt; Mystery, Thriller &amp; Suspense &gt; Cozy Mystery</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>When the groom's grandfather's gold signet ring disappears an hour before the Wexford and Adair wedding at the Tern Harbor inn, wedding planner Winnie Dorsey has to find it before the reception starts. By midnight the best man is dead on the boathouse dock, the police call it a fall, and Winnie does not believe it. Her search runs through a nervous bridal party, a jealous florist, a harbor full of gossip and Jonah Pell, the harbor master who has been her favorite irritation since high school and who is now the only person willing to check the tide logs with her. The book is a sweet, funny cozy romantic mystery with no explicit sexual content, no profanity and no on-page violence. The clues are fair, the romance is slow and earned, and the ending solves the murder, saves the wedding and leaves Winnie and Jonah with a first date. It is Book 1 of a series set in Tern Harbor, with a recurring cast of vendors, inn staff and a boat-shop cat.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>text-only</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $2.79 per sale before any delivery fee.</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>about 200 to 225 pages (estimate, about 275 words a page)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>55,000 to 62,000 words</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Adult readers of romantic comedy and cozy mysteries who read on Kindle Unlimited, mostly women aged 28 to 55 who want a mystery with a love story and a happy ending.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1. The Ring Goes Missing: Winnie finds the signet ring gone one hour before the ceremony.
-2. The Harbor Master Says No: Jonah refuses to help, then changes his mind when the best man's car turns up at the dock.
-3. Something Borrowed: Winnie interviews the bridal party and finds three people with a reason to lie.
-4. The Boathouse at Midnight: the best man is found dead on the boathouse dock.
-5. Tide Tables and Lies: Winnie and Jonah compare the tide logs with the coroner's report.
-6. The Florist's Secret: a jealous florist and an old feud complicate the timeline.
-7. Rehearsal Dinner: a toast reveals a debt and a motive.
-8. Slow Dancing in the Rain: a quiet evening turns the banter into something real.
-9. The Ring Is Found: the signet ring turns up somewhere nobody expected.
-10. Vows: the killer is exposed and the wedding goes on.
-11. First Date: a short epilogue, a first date and a hook for Book 2.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Nobody Brings a Shovel to a Wedding: A Cozy Romantic Mystery in Tern Harbor, Book 1
-Ring Bearer: A Cozy Romantic Mystery
-Something Borrowed, Someone Buried: A Tern Harbor Mystery</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>cozy romantic mystery
-romantic comedy mystery novel
-wedding planner cozy mystery
-small town cozy mystery romance
-funny cozy mystery kindle unlimited
-sweet romantic mystery series
-cozy mystery romance book one</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>ESTIMATE. No sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045, the midpoint of $0.0040 to $0.0045 for 2026. Monthly revenue = sales x $2.79 + KENP pages x $0.0045. Conservative: 10 sales and 1,500 KENP pages a month, about $35. Mid: 25 sales and 6,000 pages, about $97. Optimistic (series of three or more books): 60 sales and 15,000 pages, about $235.</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Crowded category with large publishers. Differentiate with the wedding-planner hook and a clear series arc.
-AI-drafted romance can read flat. The chemistry and dialogue need a human editor before upload.
-Cozy mystery clues must be fair and the timeline must hold. Run a timeline check against the tide logs in review.
-Cozy Mystery is adjacent to Women Sleuths, which the 2026-10-17 topic used. Confirm the owner is comfortable with this pairing.
-No sales data for this premise. Test one price before committing to Book 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Kindle Store &gt; Kindle eBooks &gt; Crafts, Hobbies &amp; Home &gt; Crafts | Kindle Store &gt; Kindle eBooks &gt; Travel</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Many adults who want a travel journal stop after the first page because they believe they cannot draw. Pocket Sketchbook is a 30-day beginner's guide to sketching on trips. It teaches the few skills that make a quick drawing of a street, a cafe or a harbor recognizable: seeing shapes before details, drawing simple buildings with one or two vanishing points, sketching people as quick gestures, and adding color in ten minutes with a limited palette. Each chapter ends with a practice task of 15 to 20 minutes that can be done at home before the trip. The book is practical rather than a talent test, and it makes no medical, financial or legal claims. Because it is text-only, every drawing step is described in plain words, and every technique claim is checked against a named source listed in the metadata before publication. Destination facts are left out so the book does not go stale.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>text-only</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>70% tier (list price between $2.99 and $9.99). About $3.49 per sale before any delivery fee.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>about 55 to 65 Kindle pages (estimate, from 12,000 to 14,000 words at about 220 words a page)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>12,000 to 14,000 words</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Adults aged about 35 to 70 who travel, want a sketching habit and believe they cannot draw. They buy Kindle guides for a hobby and want something they can read before a trip and keep in a bag.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>1. Why Travel Sketching Works: the goal is a memory, not a masterpiece.
-2. Pack Light: a pen, a small brush, a travel palette and a pocket sketchbook.
-3. Ten Lines a Day: warm-up drills for line, shape and proportion.
-4. Seeing Before Drawing: contour and gesture drawing, step by step.
-5. Buildings Without a Ruler: simple perspective with one and two vanishing points.
-6. People in Motion: sketching figures as quick shapes and capturing a street scene.
-7. Color in Ten Minutes: a limited palette and quick washes.
-8. Writing in the Margins: captions, dates and simple travel journaling.
-9. Sketching in Public: onlookers, weather and time limits.
-10. Thirty Days Before the Trip: a practice plan and a final review sheet.</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Pocket Sketchbook: A Beginner's 30-Day Guide to Drawing on the Road
-Draw Where You Are: Travel Sketching for Adults Who Think They Can't Draw
-The Little Travel Sketchbook: Thirty Days of Simple Drawing and Color</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>travel sketching for beginners
-sketchbook guide for adult beginners
-travel journaling drawing guide
-learn to sketch on vacation
-beginner drawing guide for adults
-pocket sketchbook drawing tips
-drawing for adults who cannot draw</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>ESTIMATE. No Kindle sales data was verified; these are planning assumptions. Price and royalty come from the plan. The per-page KENP rate is a third-party estimate of $0.0045 (midpoint of $0.0040 to $0.0045 for 2026). Monthly revenue = sales x $3.49 + KENP pages x $0.0045. Conservative: 8 sales and 1,000 KENP pages a month, about $32. Mid: 20 sales and 4,000 pages, about $88. Optimistic (a follow-up destination title): 45 sales and 10,000 pages, about $202.</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Text-only means drawing steps are explained in words without example images. The instructions must be clear enough to follow without pictures; a figure-based edition would need a different format.
-The urban sketching space has established named series. Do not use series names or the Urban Sketching Handbook title.
-Technique claims need named sources in metadata.json. Any unsourced technique claim is removed.
-Amazon Best Sellers and KDP help pages were not available, so the niche has no direct Kindle sales data.
-Destination facts are excluded to avoid stale information.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kindle-1: 2 topics for 2026-10-19
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -880,6 +880,233 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Staged for Love: A Larkspur Lake Romantic Comedy, Book 1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Romantic Comedy | Kindle Store &gt; Kindle eBooks &gt; Romance &gt; Contemporary &gt; Small Town</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tessa Marsh inherits her late uncle's home-staging business in Larkspur Lake, Wisconsin, a small resort town that comes alive every summer when the lake cottages go on the market. On the first morning, she pulls into the Birch Street cottage and finds a rival stager already unloading a cream sofa on the lawn, the same sofa she has brought for the same open house. The rival is Owen Reyes, a local realtor who has been quietly using her uncle's old props in his own listings. The two agree to split the Birch Street job and immediately start to bicker over every lamp, rug and throw pillow. As the summer goes on, their rivalry turns into a partnership, and then into something neither of them planned. Tessa has to decide whether to sell the business and go back to Chicago or to stay and build something of her own. The story is witty, warm and romantic, with a close-knit lake-town cast, a family dog and a clear happy ending. It has no explicit sexual content, no profanity and no on-page violence.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>text-only</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>70% (US list price between $2.99 and $12.99). About $2.69 per sale after the delivery fee (estimate: a 1 MB file at $0.15 per MB).</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>about 230 to 250 pages (estimate)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>55,000 to 62,000 words</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Adult readers of contemporary romantic comedy, mostly women 28 to 55, who read on Kindle Unlimited and want a witty, warm love story with a clear happy ending and a strong sense of place.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Moving Day: Tessa Marsh arrives in Larkspur Lake to run her late uncle's staging business and finds a rival's truck in the drive.
+The Sofa Standoff: Tessa and Owen Reyes both show up at the Birch Street cottage with the same cream sofa.
+Terms of Truce: they agree to split the Birch Street listing and argue over every lamp and rug.
+Open House Disaster: a staging mishap in front of buyers forces them to work together in public.
+Borrowed Lamps: Tessa finds her uncle's old props in Owen's storage unit and asks why.
+Dock Lights: a late-night talk on the public pier changes the tone between them.
+The Competing Listing: a buyer chooses between their two proposals, and the stakes rise.
+Rain Day: a storm leaks through the cottage roof, and they spend a long night fixing the living room.
+Her Uncle's Ledger: Tessa reads the notebook he left behind and learns that Owen was his partner.
+Summer Fair: the whole town takes sides, and Tessa has to stand up for the business she has built.
+Closing Day and the Epilogue: Tessa chooses Larkspur Lake and tells Owen the truth, and the last scene sets up Book 2.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Staged for Love
+A Larkspur Lake Romantic Comedy, Book 1
+Closing Day at Larkspur Lake
+A Romantic Comedy
+The Sofa Standoff
+A Small-Town Romantic Comedy</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>romantic comedy novel
+contemporary romantic comedy
+lake town romance novel
+home staging romantic comedy
+rival romance kindle unlimited
+clean romantic comedy for adults
+romantic comedy book 1 series</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>ESTIMATE. No sales data was verified. These are planning assumptions, not sourced figures.
+Price $3.99. The 70% royalty is about $2.69 per sale (0.70 x ($3.99 minus about $0.15 delivery fee for a 1 MB file)).
+KENP is about $0.00517 per page read (August 2026, third-party estimate, not an Amazon figure).
+Conservative: 8 sales and 1,500 KENP pages a month, about $29 a month. Mid: 25 sales and 6,000 pages, about $98. Optimistic (3 or more books in the series): 60 sales and 15,000 pages, about $239.
+Formula: sales x $2.69 + KENP pages x $0.00517.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Crowded romance shelf: differentiate with the home-staging business, the rival setup and a strong cover.
+AI-drafted romance can read flat: a human editor must work on dialogue and chemistry before upload.
+Small Town is the same subgenre as The Bakery on Cutter Street (used 2026-10-18). The premise, setting, business and cast must stay clearly different.
+Small Town was used by a topic selected in the last 7 days. Romance has no other valid pair of pool categories, so it is used here (rule exception, recorded in the run log).
+The 70% band ceiling ($12.99) and the $0.15 per MB delivery fee come from one third-party source. Confirm both on KDP's site before pricing.
+The KENP per-page rate is a third-party estimate ($0.00517 for August 2026). Confirm it before forecasting page reads.
+The title may collide with existing books. Check the KDP search before upload.
+The book is AI-written text and must be disclosed to KDP as AI-generated content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ten Stitches, Thirty Days: A Beginner's Hand Embroidery Guide</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Crafts, Hobbies &amp; Home &gt; Crafts | Kindle Store &gt; Kindle eBooks &gt; Self-Help &gt; Personal Transformation</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ten Stitches, Thirty Days teaches adults who are new to hand embroidery one stitch at a time. Readers learn which tools and fabrics to buy, how to transfer a design onto fabric, and ten core stitches: running, backstitch, straight, stem, split, chain, satin, French knot, lazy daisy and blanket stitch. Each stitch has numbered steps, a short list of common mistakes and a 15-minute practice session in a thirty-day schedule that builds gradually. The book ends with a hoop sampler that uses all ten stitches as a finished project. The self-help angle is steady, low-pressure practice and a routine that fits a busy week. It makes no health or mood promises. This is general craft instruction, not professional advice, and every stitch name and step is checked against a named source.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>text-only</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>70% (US list price between $2.99 and $12.99). About $3.39 per sale after the delivery fee (estimate: a 1 MB file at $0.15 per MB).</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>about 65 to 75 pages (estimate)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>14,000 to 17,000 words</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Adults 25 to 65 who want a calm, hands-on hobby, gift makers, and people who tried embroidery once and want a clear, patient starting point.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Before the Needle: the tools, fabrics, hoops and threads a beginner needs.
+Transferring a Design: tracing methods, water-soluble markers and choosing fabric.
+Running, Backstitch and Straight Stitch: the basic lines and how to keep them even.
+Stem, Split and Chain: curves, outlines and textured lines.
+Satin and Long-and-Short: filling shapes smoothly.
+French Knots, Lazy Daisy and Blanket Stitch: dots, petals and finished edges.
+Fixing Mistakes Without Tears: unpicking, tension and puckering.
+Thirty Days of Practice: the daily schedule, with one short session per day.
+The Hoop Sampler: a finished project that uses all ten stitches.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Ten Stitches, Thirty Days
+A Beginner's Hand Embroidery Guide
+Stitch by Stitch
+Thirty Days of Beginner Hand Embroidery
+The Hoop Sampler
+Ten Core Stitches for Beginners</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>beginner hand embroidery guide
+embroidery stitches for beginners
+hand embroidery book for adults
+embroidery stitch guide 30 days
+learn embroidery at home
+embroidery hoop sampler project
+beginner embroidery stitch book</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>ESTIMATE. No sales data was verified. These are planning assumptions, not sourced figures.
+The only book in the top 10 of Amazon's July 2026 beginner embroidery results was estimated at about 1,000 units a month (asinsight, third-party estimate, not Amazon data).
+Price $4.99. The 70% royalty is about $3.39 per sale (0.70 x ($4.99 minus about $0.15 delivery fee for a 1 MB file)).
+Practical guides usually sell outright, so KENP is not counted.
+Conservative: 8 sales a month, about $27. Mid: 20 sales, about $68. Optimistic (a series of 3 or more): 45 sales, about $153.
+Formula: sales x $3.39.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Stitch instructions must be checked against named references while drafting. Errors would be obvious to experienced stitchers.
+Crowded stitch-book market: the 30-day structure and the hoop sampler project are the differentiators.
+The self-help angle must not make health, mood or stress-relief claims unless a source supports them.
+Personal Transformation was used by a topic selected in the last 7 days. Crafts needs a second category from the pool, so it is used here (rule exception, recorded in the run log).
+The title may collide with existing books. Check the KDP search before upload.
+The book is AI-written text and must be disclosed to KDP as AI-generated content.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kindle-1: 2 topics for 2026-10-20
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZeVJcyf7XvKRRCE6AUkLk
</commit_message>
<xml_diff>
--- a/ebooks-Raw/topics-list.xlsx
+++ b/ebooks-Raw/topics-list.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1107,6 +1107,218 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Juniper Pell and the Humming Key: A Bedtime Chapter Book for Ages 6 to 9</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Children's eBooks &gt; Early Chapter Books | Kindle Store &gt; Kindle eBooks &gt; Children's eBooks &gt; Bedtime Stories</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>When eight-year-old Juniper Pell finds a brass key on her porch step, it hums softly whenever she holds it near the old Hollow Oak Library, which closed last winter. With her friend Benji and her four-year-old brother Otis tagging along, Juniper follows the humming through a small door behind the fiction shelves and into a library that is quiet, dim and full of glowing books. The library cat, Pepper, leads them through corridors where stories are kept like lanterns, and a book with blank pages begins to write itself once Juniper reads its first line aloud. The town's bedtime songs have gone missing, and only the key can bring them back. Juniper learns that the librarian, Ms. Hart, knew the key's history all along. The story is gentle and warm, with short sentences, a clear problem and a positive ending. It contains no violence and nothing frightening, and each chapter ends with a reason to turn the page.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>text-only</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>70% (US list price between $2.99 and $9.99). About $2.64 per sale after the delivery fee (estimate: a 1 MB file at $0.15 per MB).</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>about 70 to 85 pages (estimate)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>10,000 to 13,000 words</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Children aged 6 to 9 reading on their own (reading level grade 2 to 4), and parents and grandparents reading aloud at bedtime. Mostly US Kindle and Kindle Unlimited readers.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>The Humming Key: Juniper finds a brass key on her porch step that hums when she holds it.
+Closed for Winter: Juniper and Benji walk to the Hollow Oak Library and find a sign that says closed.
+A Door in the Reading Room: the key fits a small door behind the fiction shelves.
+Pepper Knows the Way: the library cat leads them down a corridor of glowing books.
+The Book That Writes Back: a book with blank pages starts a story when Juniper reads its first line aloud.
+Otis Follows: the little brother sneaks in and wanders among the picture books.
+The Missing Lullabies: the town's bedtime songs have gone quiet, and the key is the only way to bring them back.
+Ms. Hart's Secret: the librarian explains the key's history and why the library needed it.
+The Quiet Stacks: Juniper reads aloud in the dim aisles to light the way home.
+Lights On, Key Asleep: the three children reach home before bedtime, and the key rests on the windowsill.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Juniper Pell and the Humming Key
+A Bedtime Chapter Book for Ages 6 to 9
+The Humming Key
+A Juniper Pell Adventure, Book 1
+Juniper Pell and the Library After Dark
+A Gentle Chapter Book for Young Readers</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>chapter books for kids ages 6 to 9
+bedtime chapter book for early readers
+chapter book for second graders
+gentle library adventure for kids
+read aloud chapter book at bedtime
+kids mystery chapter book series
+early chapter book for young readers</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>ESTIMATE: about 5 to 15 paid sales per month in the first year at $3.99, with some Kindle Unlimited page reads. Basis: KDPEasy rates demand High and competition High for this niche (site estimate, not sales data). Royalty about $2.64 per sale (estimate). Income depends on a series; a single title is unlikely to pay much on its own.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Competition is rated High on KDPEasy (site estimate); the hook must be strong on the cover and in the sales copy.
+Reading level must pass the grade 2 to 4 readability check in guide section 13. Vocabulary can drift upward in a mystery, so the check may need a revision pass.
+Pairing a chapter book with the Bedtime Stories category is a judgment call. It is a valid pool pair, but the owner may prefer a different reading of the shelf.
+A single book earns little. The series plan (Book 2 and later) matters for income.
+The library setting must stay gentle. Keep the dim stacks and the dark moments mild, with no frightening scenes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Selected</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The Open Road Plan: A Workbook for Retirees Planning Their First Long Road Trip</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Kindle Store &gt; Kindle eBooks &gt; Self-Help &gt; Aging or Retirement | Kindle Store &gt; Kindle eBooks &gt; Travel</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Many retirees dream of a long road trip and never start planning it. The Open Road Plan is a step-by-step workbook that helps you turn that dream into a route, a daily pace, a budget and a packing list. Each chapter asks you to write your own answers in short prompts and answer blocks: why you want to go, what kind of trip you enjoy, how far you want to drive each day, which scenic roads and rest stops fit your route, where you will stay, and what a trip of this length tends to cost. The workbook explains each planning step in plain language and points to named public sources for route, park and road-safety facts, so you can check details before you go. It finishes with a packing checklist and a trip log you fill in on the road. It is written for practical planning only and includes the general-information disclaimer required for practical guides.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>workbook</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>70% (US list price between $2.99 and $9.99). About $2.65 per sale after the delivery fee (estimate: a 1 MB file at $0.15 per MB).</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>about 125 to 150 pages (estimate, including answer blocks)</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>13,000 to 15,000 words</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Retirees aged 60 to 75 planning their first long road trip, and couples or solo travelers who like to plan at the kitchen table. Reader age 55 to 75. Mostly US Kindle and Kindle Unlimited readers who want a practical, printable-style workbook they can complete on a tablet.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Why Now: name your reasons for the trip and set a realistic start date.
+Your Travel Style: decide your pace, comfort level and who is coming along.
+Choosing the Route: sketch a loop, pick scenic roads and mark possible rest stops.
+Daily Pacing: plan driving hours, breaks and stops for each day of the trip.
+Stays and Stops: plan lodging, reservations and backup options for each night.
+The Trip Budget: list the main costs, add a buffer and track your numbers.
+Road Readiness: check the vehicle, documents, contacts and a simple emergency plan.
+Packing and the Trip Log: use the checklists and fill in a log while you travel.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>The Open Road Plan
+A Workbook for Retirees Planning Their First Long Road Trip
+Retirement Road Trip Workbook
+Plan Your Route, Pace and Budget
+Hit the Road After Retirement
+A Planning Workbook for Your First Big Trip</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>retirement road trip planner workbook
+road trip planning workbook for retirees
+retiree travel planning guide
+first long road trip planner
+senior road trip itinerary workbook
+travel planning workbook for seniors
+retirement travel budget workbook</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>ESTIMATE: about 3 to 10 paid sales per month in the first year at $3.99, with some Kindle Unlimited page reads. Basis: Amazon listings for senior road-trip and retirement-travel titles show active competition, but no sales or rank data was readable. Royalty about $2.65 per sale (estimate).</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Crowded shelf: Route 66 and senior road-trip guides already sell on Amazon. The workbook format and answer blocks are the differentiator.
+Facts go stale. Fuel prices, park fees, road closures and lodging rules change, so each figure needs a dated, named source and a check before publishing.
+Budget chapter can drift into financial advice. Keep it to general planning with the disclaimer.
+Safety chapter can drift into medical advice. Keep it to general road readiness and planning, with no health claims.
+Workbooks need at least 10 answer blocks, and check_book.py counts them. Each block needs three lines to write on.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>